<commit_message>
Changed the window name
</commit_message>
<xml_diff>
--- a/Rubric.xlsx
+++ b/Rubric.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSU\dev5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xinar\source\repos\Dev5\Red-2604\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4581CF42-ABC0-4AA9-AB57-A5CE013C34AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B36E6A1-E29D-43A0-ACBF-409E20BDB0F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7476" yWindow="2256" windowWidth="23040" windowHeight="13560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Info" sheetId="1" r:id="rId1"/>
@@ -1918,12 +1918,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="50.6640625" customWidth="1"/>
+    <col min="1" max="3" width="50.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="19.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -1934,7 +1934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="29" t="s">
         <v>95</v>
       </c>
@@ -1945,33 +1945,33 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C3" s="13" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C4" s="13" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C5" s="13" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C6" s="13" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C7" s="24"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C8" s="23"/>
     </row>
-    <row r="9" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.4">
       <c r="A9" s="17" t="s">
         <v>3</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="18">
         <v>2851</v>
       </c>
@@ -1993,28 +1993,28 @@
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C11" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C12" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C13" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C15" s="1"/>
     </row>
-    <row r="17" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.4">
       <c r="A17" s="17" t="s">
         <v>5</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="25" t="s">
         <v>93</v>
       </c>
@@ -2050,16 +2050,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{976D0730-B5D0-49E5-8631-8CC13B9FE765}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:G82"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="83.44140625" customWidth="1"/>
-    <col min="2" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" customWidth="1"/>
-    <col min="5" max="7" width="9.109375" hidden="1" customWidth="1"/>
-    <col min="11" max="13" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="83.453125" customWidth="1"/>
+    <col min="2" max="3" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" customWidth="1"/>
+    <col min="5" max="7" width="9.08984375" hidden="1" customWidth="1"/>
+    <col min="11" max="13" width="9.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="30" t="s">
         <v>34</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="34" t="s">
         <v>74</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>69</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="12" t="s">
         <v>72</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="12" t="s">
         <v>73</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
         <v>80</v>
       </c>
@@ -2145,14 +2145,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="34" t="s">
         <v>83</v>
       </c>
       <c r="B7" s="34"/>
       <c r="C7" s="33"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
         <v>68</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
         <v>86</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
         <v>85</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
         <v>84</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>87</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="12" t="s">
         <v>33</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="12" t="s">
         <v>32</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
         <v>25</v>
       </c>
@@ -2240,14 +2240,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="34" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="34"/>
       <c r="C16" s="33"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="12" t="s">
         <v>81</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
         <v>47</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
         <v>48</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
         <v>91</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
         <v>90</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
         <v>43</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="12" t="s">
         <v>45</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="12" t="s">
         <v>40</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
         <v>41</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="12" t="s">
         <v>44</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="12" t="s">
         <v>46</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
         <v>37</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="12" t="s">
         <v>88</v>
       </c>
@@ -2390,14 +2390,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="34" t="s">
         <v>65</v>
       </c>
       <c r="B30" s="34"/>
       <c r="C30" s="33"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="12" t="s">
         <v>70</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="12" t="s">
         <v>76</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="12" t="s">
         <v>75</v>
       </c>
@@ -2430,14 +2430,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="34" t="s">
         <v>78</v>
       </c>
       <c r="B34" s="34"/>
       <c r="C34" s="33"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="12" t="s">
         <v>79</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="12" t="s">
         <v>71</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:3" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="32" t="s">
         <v>39</v>
       </c>
@@ -2472,16 +2472,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
     </row>
-    <row r="40" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:3" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="36" t="s">
         <v>49</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
         <v>26</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
         <v>58</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
         <v>63</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="11" t="s">
         <v>67</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
         <v>20</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="11" t="s">
         <v>11</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:3" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="32" t="s">
         <v>61</v>
       </c>
@@ -2571,13 +2571,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:2" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="36" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="46"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="12" t="s">
         <v>28</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="12" t="s">
         <v>29</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="12" t="s">
         <v>36</v>
       </c>
@@ -2601,7 +2601,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="12" t="s">
         <v>31</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
         <v>89</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="12" t="s">
         <v>77</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
         <v>82</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="12" t="s">
         <v>64</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:2" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="32" t="s">
         <v>66</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:2" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="36" t="s">
         <v>53</v>
       </c>
@@ -2658,13 +2658,13 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" s="34" t="s">
         <v>51</v>
       </c>
       <c r="B63" s="42"/>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" s="11" t="s">
         <v>59</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="11" t="s">
         <v>13</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="11" t="s">
         <v>60</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="11" t="s">
         <v>30</v>
       </c>
@@ -2696,13 +2696,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="34" t="s">
         <v>54</v>
       </c>
       <c r="B68" s="42"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="11" t="s">
         <v>55</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="11" t="s">
         <v>56</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>19</v>
       </c>
@@ -2726,13 +2726,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="34" t="s">
         <v>52</v>
       </c>
       <c r="B72" s="42"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
         <v>12</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" s="11" t="s">
         <v>17</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" s="11" t="s">
         <v>16</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" s="11" t="s">
         <v>57</v>
       </c>
@@ -2764,13 +2764,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="19.8" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:2" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A79" s="44" t="s">
         <v>21</v>
       </c>
       <c r="B79" s="43"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" s="40" t="s">
         <v>24</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" s="40" t="s">
         <v>23</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" s="40" t="s">
         <v>22</v>
       </c>

</xml_diff>